<commit_message>
working heuristic for MCV. Entire set missing vaccine price issue
</commit_message>
<xml_diff>
--- a/Heuristic/data/real/start_generator.xlsx
+++ b/Heuristic/data/real/start_generator.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/Heuristic/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/Heuristic/data/real/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B85D085A-19C2-43D8-BE5B-5625CEB2C3E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{B85D085A-19C2-43D8-BE5B-5625CEB2C3E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD067E41-F37B-44ED-B066-C1D5CFD38FEB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{11746B91-1220-436F-8126-EEF4BA69D2A9}"/>
   </bookViews>
@@ -19,7 +19,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">antigen_demand_80_20_2_scenario!$A$1:$D$25</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1478,7 +1491,7 @@
         <v>278836000</v>
       </c>
       <c r="F8">
-        <f t="shared" ref="F8:F9" si="2">SUM(C8:E8)</f>
+        <f>SUM(C8:E8)</f>
         <v>837500100</v>
       </c>
     </row>
@@ -1491,15 +1504,15 @@
         <v>26052200</v>
       </c>
       <c r="D9">
-        <f t="shared" ref="D9:E9" si="3">D4</f>
+        <f t="shared" ref="D9:E9" si="2">D4</f>
         <v>26626400</v>
       </c>
       <c r="E9">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>25785400</v>
       </c>
       <c r="F9">
-        <f t="shared" si="2"/>
+        <f>SUM(C9:E9)</f>
         <v>78464000</v>
       </c>
     </row>

</xml_diff>